<commit_message>
Fix blank-page bug in Validacion Maquina Segura PDFs, compact to 6 pages
The 28-page PDFs weren't actually missing content -- fitToHeight=0 let
gnumeric's automatic page-break placement land right after dense
sections, leaving the remainder of a tall near-empty row (signature
block, the 20-row-tall photo merge) as its own mostly-blank page.
Fixed by setting an explicit fitToHeight per sheet (EHS=2, SME=4)
instead of auto, which forces gnumeric to compute one scale factor that
distributes real content evenly across exactly that many pages --
6 pages total per station, zero blank pages, full page width, legible
text. Applied to all 16 stations' real .xlsx print setup and
regenerated all 16 PDFs.
</commit_message>
<xml_diff>
--- a/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Ampseal_Attach_Gecko.xlsx
+++ b/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Ampseal_Attach_Gecko.xlsx
@@ -6281,7 +6281,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="1" fitToHeight="2" fitToWidth="1"/>
   <headerFooter alignWithMargins="0">
     <oddHeader/>
     <oddFooter>&amp;L&amp;16 &amp;K00000016-HS80-8000-00010-I / 16-HS20-8000-00010&amp;R&amp;16 Tiempo de retención en el punto de origen: 3 años_x000a_Tiempo de retención en archivo muerto: N/A_x000a_Medio de registro :Electrónico</oddFooter>
@@ -12187,7 +12187,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="1.6975" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="1" fitToHeight="4" fitToWidth="1"/>
   <headerFooter alignWithMargins="0">
     <oddHeader/>
     <oddFooter>&amp;L&amp;14 &amp;K00000016-HS80-8000-00010-I / 16-HS20-8000-00010&amp;RTiempo de retención en el punto de origen: 3 años_x000a_Tiempo de retención en archivo muerto: N/A_x000a_Medio de registro :Electrónico</oddFooter>

</xml_diff>

<commit_message>
Ajustar PDFs de Validacion Maquina Segura a 3 paginas en Carta estandar
Cambia fitToHeight de EHS=2/SME=4 (6 paginas) a EHS=1/SME=2 (3 paginas),
manteniendo tamaño de papel Carta (Letter) en lugar de Tabloid para
impresión normal de oficina. Verificado visualmente sin páginas en blanco.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PtjxNEToLwFA6ZBpe5Zyeg
</commit_message>
<xml_diff>
--- a/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Ampseal_Attach_Gecko.xlsx
+++ b/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Ampseal_Attach_Gecko.xlsx
@@ -6281,7 +6281,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="1" fitToHeight="2" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="1" fitToHeight="1" fitToWidth="1"/>
   <headerFooter alignWithMargins="0">
     <oddHeader/>
     <oddFooter>&amp;L&amp;16 &amp;K00000016-HS80-8000-00010-I / 16-HS20-8000-00010&amp;R&amp;16 Tiempo de retención en el punto de origen: 3 años_x000a_Tiempo de retención en archivo muerto: N/A_x000a_Medio de registro :Electrónico</oddFooter>
@@ -12187,7 +12187,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="1.6975" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="1" fitToHeight="4" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="1" fitToHeight="2" fitToWidth="1"/>
   <headerFooter alignWithMargins="0">
     <oddHeader/>
     <oddFooter>&amp;L&amp;14 &amp;K00000016-HS80-8000-00010-I / 16-HS20-8000-00010&amp;RTiempo de retención en el punto de origen: 3 años_x000a_Tiempo de retención en archivo muerto: N/A_x000a_Medio de registro :Electrónico</oddFooter>

</xml_diff>

<commit_message>
Cambiar PDFs de Validacion Maquina Segura a A4 vertical (tamaño típico MX)
Cambia orientación de horizontal/Carta a vertical/A4 (el tamaño típico
usado en México), fitToHeight EHS=1/SME=2, y elimina los saltos de
página manuales heredados de la plantilla (filas 57/107 en Check List
SME) que causaban páginas en blanco adicionales al cambiar de formato.
Resultado: 3 páginas por estación, A4 vertical, sin páginas en blanco.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PtjxNEToLwFA6ZBpe5Zyeg
</commit_message>
<xml_diff>
--- a/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Ampseal_Attach_Gecko.xlsx
+++ b/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Ampseal_Attach_Gecko.xlsx
@@ -6281,7 +6281,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="1" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter alignWithMargins="0">
     <oddHeader/>
     <oddFooter>&amp;L&amp;16 &amp;K00000016-HS80-8000-00010-I / 16-HS20-8000-00010&amp;R&amp;16 Tiempo de retención en el punto de origen: 3 años_x000a_Tiempo de retención en archivo muerto: N/A_x000a_Medio de registro :Electrónico</oddFooter>
@@ -6290,9 +6290,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <rowBreaks count="1" manualBreakCount="1">
-    <brk id="38" min="0" max="22" man="1"/>
-  </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -12187,7 +12184,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="1.6975" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="1" fitToHeight="2" fitToWidth="1"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="2" fitToWidth="1"/>
   <headerFooter alignWithMargins="0">
     <oddHeader/>
     <oddFooter>&amp;L&amp;14 &amp;K00000016-HS80-8000-00010-I / 16-HS20-8000-00010&amp;RTiempo de retención en el punto de origen: 3 años_x000a_Tiempo de retención en archivo muerto: N/A_x000a_Medio de registro :Electrónico</oddFooter>
@@ -12196,10 +12193,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <rowBreaks count="2" manualBreakCount="2">
-    <brk id="57" min="0" max="22" man="1"/>
-    <brk id="107" min="0" max="22" man="1"/>
-  </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Dejar en B91 solo dispositivos de seguridad (quitar switches generales)
Se quitan del bloque de interlocks/sensores (B91) las fotos que no son
estrictamente "dispositivo de seguridad": switch principal/sistema FRL
y power switch (son controles de energia/aire, no dispositivos de
seguridad) y la foto del piston del cortador (no muestra un dispositivo).
B91 queda solo con: cortina de seguridad (donde aplica), paro de
emergencia, y switch/interlock de la cortina (Gecko). Se regeneraron
los 16 PDF individuales, el merge de 48 paginas y el merge de solo
pagina 3.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PtjxNEToLwFA6ZBpe5Zyeg
</commit_message>
<xml_diff>
--- a/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Ampseal_Attach_Gecko.xlsx
+++ b/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Ampseal_Attach_Gecko.xlsx
@@ -1784,7 +1784,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" l="34082" t="29556" r="36328" b="57813"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -1828,7 +1828,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -1877,7 +1877,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1921,7 +1921,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -1967,7 +1967,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" l="34082" t="29556" r="36328" b="57813"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -2004,13 +2004,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2029,13 +2032,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2105,31 +2111,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>11</col>
-      <colOff>95250</colOff>
-      <row>98</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <ext cx="4953000" cy="5876925"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="11" name="Image 11" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>

</xml_diff>

<commit_message>
Quitar por completo fotos de guardas, dejar solo dispositivos de seguridad
Se elimina cualquier foto de guarda/mascara/feeder/gabinete de ambos
bloques de fotos (B71 y B91). Ambos bloques quedan con el mismo
contenido: solo dispositivos de seguridad (cortina de presencia,
switch/interlock de seguridad, paro de emergencia), respetando la
excepcion de 9 estaciones sin foto de cortina. Se regeneraron los 16
PDF, el merge de 48 paginas y el merge de solo pagina 3.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PtjxNEToLwFA6ZBpe5Zyeg
</commit_message>
<xml_diff>
--- a/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Ampseal_Attach_Gecko.xlsx
+++ b/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Ampseal_Attach_Gecko.xlsx
@@ -1784,7 +1784,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" l="34082" t="29556" r="36328" b="57813"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -1828,7 +1828,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -1877,7 +1877,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1921,7 +1921,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -1967,7 +1967,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" l="34082" t="29556" r="36328" b="57813"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -1997,23 +1997,20 @@
       <row>70</row>
       <rowOff>95250</rowOff>
     </from>
-    <ext cx="4953000" cy="6496050"/>
+    <ext cx="4953000" cy="6915150"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2025,23 +2022,45 @@
       <row>70</row>
       <rowOff>95250</rowOff>
     </from>
-    <ext cx="4953000" cy="3971925"/>
+    <ext cx="4953000" cy="4800600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="7" name="Image 7" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>95250</colOff>
+      <row>80</row>
+      <rowOff>95250</rowOff>
+    </from>
+    <ext cx="4953000" cy="2781300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2056,11 +2075,11 @@
     <ext cx="4953000" cy="6915150"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2081,11 +2100,11 @@
     <ext cx="4953000" cy="4800600"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2106,11 +2125,11 @@
     <ext cx="4953000" cy="2781300"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>

</xml_diff>

<commit_message>
Agregar paro de emergencia y switch genéricos también en las 8 estaciones Gecko
Se agregan en el espacio libre del bloque B71 (debajo de las 2 fotos
nuevas de jaula/bisagra), sin tocar el bloque B91 (cortina+switch+paro
de familia). Verificado visualmente sin traslapes en los 2 casos
(Gecko con/sin cortina).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PtjxNEToLwFA6ZBpe5Zyeg
</commit_message>
<xml_diff>
--- a/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Ampseal_Attach_Gecko.xlsx
+++ b/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Ampseal_Attach_Gecko.xlsx
@@ -2146,6 +2146,56 @@
         <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>95250</colOff>
+      <row>80</row>
+      <rowOff>95250</rowOff>
+    </from>
+    <ext cx="4381500" cy="4333875"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>95250</colOff>
+      <row>80</row>
+      <rowOff>95250</rowOff>
+    </from>
+    <ext cx="4381500" cy="3305175"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>

</xml_diff>

<commit_message>
Mover paro/switch genéricos de Gecko a la celda de abajo (B91)
Se quitan de B71 (que vuelve a tener solo las 2 fotos propias de
Gecko: jaula y bisagra) y se agregan en B91, junto con cortina+switch+
paro de familia. En las 6 estaciones con cortina solo había 1 espacio
libre en B91, así que se usa una fila extra dentro de la misma celda
combinada (B91:U106) para que quepan las 5 fotos sin traslape.
Verificado visualmente en ambos casos (con/sin cortina).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PtjxNEToLwFA6ZBpe5Zyeg
</commit_message>
<xml_diff>
--- a/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Ampseal_Attach_Gecko.xlsx
+++ b/Revalidacion Moose Scorpion Gecko/Validacion Maquina Segura/MS_Ampseal_Attach_Gecko.xlsx
@@ -2152,9 +2152,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>1</col>
+      <col>11</col>
       <colOff>95250</colOff>
-      <row>80</row>
+      <row>98</row>
       <rowOff>95250</rowOff>
     </from>
     <ext cx="4381500" cy="4333875"/>
@@ -2177,9 +2177,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>11</col>
+      <col>1</col>
       <colOff>95250</colOff>
-      <row>80</row>
+      <row>104</row>
       <rowOff>95250</rowOff>
     </from>
     <ext cx="4381500" cy="3305175"/>

</xml_diff>